<commit_message>
basic software project setup Add backlog add user stories classes defined classes made fouten verbeterd backlog verbeterd
</commit_message>
<xml_diff>
--- a/documents/backlog.xlsx
+++ b/documents/backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\intelliJ\euromoon-java\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7ABB6C1-CE86-4027-B90B-FF2D8E0BED90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C080077-1E79-47BD-9A41-9ED9652D9346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -332,7 +332,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>

</xml_diff>